<commit_message>
modified:   .DS_Store 	modified:   archive/Purchase 20260105.xlsx 	deleted:    hardware/CTL-4.3/CTL-4.3-backups/CTL-4.3-2026-01-19_090613.zip 	renamed:    hardware/CTL-4.3/CTL-4.3-backups/CTL-4.3-2026-01-19_091818.zip -> hardware/CTL-4.3/CTL-4.3-backups/CTL-4.3-2026-01-19_105947.zip 	new file:   hardware/CTL-4.3/CTL-4.3-backups/CTL-4.3-2026-01-19_110601.zip 	new file:   hardware/CTL-4.3/CTL-4.3-backups/CTL-4.3-2026-01-19_111804.zip 	new file:   hardware/CTL-4.3/CTL-4.3-backups/CTL-4.3-2026-01-19_113721.zip 	new file:   hardware/CTL-4.3/CTL-4.3-backups/CTL-4.3-2026-01-19_164107.zip 	new file:   hardware/CTL-4.3/CTL-4.3-backups/CTL-4.3-2026-01-20_112913.zip 	modified:   hardware/CTL-4.3/CTL-4.3.kicad_pcb 	modified:   hardware/CTL-4.3/CTL-4.3.kicad_sch 	modified:   hardware/CTL-4.3/bom/ibom.html 	modified:   hardware/CTL-4.3/fp-info-cache 	new file:   hardware/PS-5.1/PS-5.1-backups/PS-5.1-2026-01-19_103049.zip
</commit_message>
<xml_diff>
--- a/archive/Purchase 20260105.xlsx
+++ b/archive/Purchase 20260105.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="59">
   <si>
     <t>TOOLS</t>
   </si>
@@ -104,19 +105,19 @@
     <t>R 22 0805 1%</t>
   </si>
   <si>
-    <t>R 5.1k 1206 1%</t>
-  </si>
-  <si>
-    <t>R 10k 1206 1%</t>
-  </si>
-  <si>
-    <t>C 100nF 50V 0805 X7R 5%</t>
+    <t>R 5.1k 0805 1%</t>
+  </si>
+  <si>
+    <t>R 10k 0805 1%</t>
+  </si>
+  <si>
+    <t>C 100nF 50V 0805 X7R 10%</t>
   </si>
   <si>
     <t>C 1µF 25V 0805 X7R 10%</t>
   </si>
   <si>
-    <t>C 22pF 50V C0G</t>
+    <t>C 22pF 50V C0G 5%</t>
   </si>
   <si>
     <t>C Tantalum 22µF 10V 3528</t>
@@ -128,7 +129,7 @@
     <t>680µF 35V</t>
   </si>
   <si>
-    <t>LED</t>
+    <t>LED 1206</t>
   </si>
   <si>
     <t>D SS36 SMA</t>
@@ -141,6 +142,69 @@
   </si>
   <si>
     <t>G5V-1</t>
+  </si>
+  <si>
+    <t>R 220 1207 1%</t>
+  </si>
+  <si>
+    <t>PCB CTL</t>
+  </si>
+  <si>
+    <t>Film</t>
+  </si>
+  <si>
+    <t>PCB</t>
+  </si>
+  <si>
+    <t>Ongkir</t>
+  </si>
+  <si>
+    <t>Deskripsi</t>
+  </si>
+  <si>
+    <t>Konektor</t>
+  </si>
+  <si>
+    <t>Kabel</t>
+  </si>
+  <si>
+    <t>Komponen</t>
+  </si>
+  <si>
+    <t>Total Bahan</t>
+  </si>
+  <si>
+    <t>Selisih</t>
+  </si>
+  <si>
+    <t>CN1</t>
+  </si>
+  <si>
+    <t>XH2.5 2 + Kabel 22 25 + Heat shrink + DC022</t>
+  </si>
+  <si>
+    <t>CN2</t>
+  </si>
+  <si>
+    <t>XH2.5 2 + Kabel 22 30</t>
+  </si>
+  <si>
+    <t>CN3</t>
+  </si>
+  <si>
+    <t>XH2.5 3 + Kabel 24 25 + Heat shrink + LED</t>
+  </si>
+  <si>
+    <t>CN4</t>
+  </si>
+  <si>
+    <t>XH2.5 2 + Kabel 24 15</t>
+  </si>
+  <si>
+    <t>mirip jasa solder per point untuk PCBA (untuk 5 titik: Soket DC dan LED)</t>
+  </si>
+  <si>
+    <t>pcs</t>
   </si>
 </sst>
 </file>
@@ -765,7 +829,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -775,13 +839,28 @@
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
@@ -1054,6 +1133,20 @@
       <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="00FF2600"/>
+      <color rgb="00FF9300"/>
+      <color rgb="00FFFC00"/>
+      <color rgb="0000FA00"/>
+      <color rgb="0000FDFF"/>
+      <color rgb="000432FF"/>
+      <color rgb="00FF40FF"/>
+      <color rgb="00942092"/>
+      <color rgb="00AB7942"/>
+      <color rgb="00FFFFFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1320,7 +1413,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="5"/>
   <cols>
     <col min="2" max="2" width="46.75" customWidth="1"/>
@@ -1375,7 +1468,7 @@
       <c r="D8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="11">
         <f>SUM(E9:E17)</f>
         <v>484800</v>
       </c>
@@ -1390,7 +1483,7 @@
       <c r="D9" s="2">
         <v>98000</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="10">
         <f t="shared" ref="E9:E17" si="0">C9*D9</f>
         <v>98000</v>
       </c>
@@ -1405,7 +1498,7 @@
       <c r="D10" s="2">
         <v>198500</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="10">
         <f t="shared" si="0"/>
         <v>198500</v>
       </c>
@@ -1420,7 +1513,7 @@
       <c r="D11" s="2">
         <v>32000</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="10">
         <f t="shared" si="0"/>
         <v>32000</v>
       </c>
@@ -1435,7 +1528,7 @@
       <c r="D12" s="2">
         <v>26000</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="10">
         <f t="shared" si="0"/>
         <v>26000</v>
       </c>
@@ -1450,7 +1543,7 @@
       <c r="D13" s="2">
         <v>12500</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="10">
         <f t="shared" si="0"/>
         <v>50000</v>
       </c>
@@ -1465,7 +1558,7 @@
       <c r="D14" s="2">
         <v>6250</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="10">
         <f t="shared" si="0"/>
         <v>12500</v>
       </c>
@@ -1480,7 +1573,7 @@
       <c r="D15" s="2">
         <v>5400</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="10">
         <f t="shared" si="0"/>
         <v>21600</v>
       </c>
@@ -1495,7 +1588,7 @@
       <c r="D16" s="2">
         <v>4550</v>
       </c>
-      <c r="E16" s="3">
+      <c r="E16" s="10">
         <f t="shared" si="0"/>
         <v>18200</v>
       </c>
@@ -1510,7 +1603,7 @@
       <c r="D17" s="2">
         <v>28000</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="10">
         <f t="shared" si="0"/>
         <v>28000</v>
       </c>
@@ -1518,406 +1611,696 @@
     <row r="18" spans="3:5">
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
-      <c r="E18" s="3"/>
-    </row>
-    <row r="19" spans="1:1">
-      <c r="A19" s="1" t="s">
+      <c r="E18" s="10"/>
+    </row>
+    <row r="19" spans="3:5">
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="10"/>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="1" t="s">
+    <row r="21" spans="1:5">
+      <c r="A21" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E20" s="6">
-        <f>SUM(E21:E41)</f>
-        <v>642102</v>
-      </c>
-    </row>
-    <row r="21" spans="2:5">
-      <c r="B21" t="s">
+      <c r="E21" s="11">
+        <f>SUM(E22:E42)</f>
+        <v>644877</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5">
+      <c r="B22" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C22" s="6">
         <v>2</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D22" s="6">
         <v>120000</v>
       </c>
-      <c r="E21" s="3">
-        <f>C21*D21</f>
+      <c r="E22" s="7">
+        <f>C22*D22</f>
         <v>240000</v>
       </c>
     </row>
-    <row r="22" spans="2:5">
-      <c r="B22" t="s">
+    <row r="23" spans="2:5">
+      <c r="B23" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C23" s="6">
         <v>2</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D23" s="6">
         <v>11000</v>
       </c>
-      <c r="E22" s="3">
-        <f>C22*D22</f>
+      <c r="E23" s="7">
+        <f>C23*D23</f>
         <v>22000</v>
       </c>
     </row>
-    <row r="23" spans="2:5">
-      <c r="B23" t="s">
+    <row r="24" spans="2:5">
+      <c r="B24" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="3">
+      <c r="C24" s="7">
         <v>4</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D24" s="7">
         <v>1100</v>
       </c>
-      <c r="E23" s="3">
-        <f t="shared" ref="E23:E28" si="1">C23*D23</f>
+      <c r="E24" s="7">
+        <f t="shared" ref="E24:E29" si="1">C24*D24</f>
         <v>4400</v>
       </c>
     </row>
-    <row r="24" spans="2:5">
-      <c r="B24" t="s">
+    <row r="25" spans="2:5">
+      <c r="B25" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="3">
+      <c r="C25" s="7">
         <v>4</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D25" s="7">
         <v>10000</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E25" s="7">
         <f t="shared" si="1"/>
         <v>40000</v>
       </c>
     </row>
-    <row r="25" spans="2:5">
-      <c r="B25" t="s">
+    <row r="26" spans="2:5">
+      <c r="B26" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="3">
+      <c r="C26" s="7">
         <v>4</v>
       </c>
-      <c r="D25" s="3">
+      <c r="D26" s="7">
         <v>10000</v>
       </c>
-      <c r="E25" s="3">
+      <c r="E26" s="7">
         <f t="shared" si="1"/>
         <v>40000</v>
       </c>
     </row>
-    <row r="26" spans="2:5">
-      <c r="B26" t="s">
+    <row r="27" spans="2:5">
+      <c r="B27" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C26" s="3">
+      <c r="C27" s="7">
         <v>4</v>
       </c>
-      <c r="D26" s="3">
+      <c r="D27" s="7">
         <v>15000</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E27" s="7">
         <f t="shared" si="1"/>
         <v>60000</v>
       </c>
     </row>
-    <row r="27" spans="2:5">
-      <c r="B27" t="s">
+    <row r="28" spans="2:5">
+      <c r="B28" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C27" s="3">
+      <c r="C28" s="7">
         <v>4</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D28" s="7">
         <v>4041</v>
       </c>
-      <c r="E27" s="3">
+      <c r="E28" s="7">
         <f t="shared" si="1"/>
         <v>16164</v>
       </c>
     </row>
-    <row r="28" spans="2:5">
-      <c r="B28" t="s">
+    <row r="29" spans="2:5">
+      <c r="B29" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C28" s="3">
+      <c r="C29" s="7">
         <v>50</v>
       </c>
-      <c r="D28" s="3">
-        <v>100</v>
-      </c>
-      <c r="E28" s="3">
+      <c r="D29" s="6">
+        <v>125</v>
+      </c>
+      <c r="E29" s="7">
         <f t="shared" si="1"/>
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="29" spans="2:5">
-      <c r="B29" t="s">
+        <v>6250</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5">
+      <c r="B30" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C29" s="2">
-        <v>25</v>
-      </c>
-      <c r="D29" s="2">
-        <v>149</v>
-      </c>
-      <c r="E29" s="3">
-        <f t="shared" ref="E29:E41" si="2">C29*D29</f>
-        <v>3725</v>
-      </c>
-    </row>
-    <row r="30" spans="2:5">
-      <c r="B30" t="s">
+      <c r="C30" s="6">
+        <v>50</v>
+      </c>
+      <c r="D30" s="6">
+        <v>125</v>
+      </c>
+      <c r="E30" s="7">
+        <f t="shared" ref="E30:E43" si="2">C30*D30</f>
+        <v>6250</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5">
+      <c r="B31" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C30" s="2">
+      <c r="C31" s="6">
         <v>50</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D31" s="6">
         <v>125</v>
       </c>
-      <c r="E30" s="3">
+      <c r="E31" s="7">
         <f t="shared" si="2"/>
         <v>6250</v>
       </c>
     </row>
-    <row r="31" spans="2:5">
-      <c r="B31" t="s">
+    <row r="32" spans="2:5">
+      <c r="B32" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C31" s="2">
+      <c r="C32" s="6">
         <v>20</v>
       </c>
-      <c r="D31" s="2">
-        <v>249</v>
-      </c>
-      <c r="E31" s="3">
+      <c r="D32" s="6">
+        <v>199</v>
+      </c>
+      <c r="E32" s="7">
         <f t="shared" si="2"/>
-        <v>4980</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6">
-      <c r="B32" t="s">
+        <v>3980</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6">
+      <c r="B33" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C32" s="2">
+      <c r="C33" s="6">
         <v>20</v>
       </c>
-      <c r="D32" s="2">
+      <c r="D33" s="6">
         <v>368</v>
       </c>
-      <c r="E32" s="3">
+      <c r="E33" s="7">
         <f t="shared" si="2"/>
         <v>7360</v>
       </c>
-      <c r="F32" s="3"/>
-    </row>
-    <row r="33" spans="2:5">
-      <c r="B33" t="s">
+      <c r="F33" s="10"/>
+    </row>
+    <row r="34" spans="2:5">
+      <c r="B34" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C33" s="2">
+      <c r="C34" s="6">
         <v>25</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D34" s="6">
         <v>199</v>
       </c>
-      <c r="E33" s="3">
+      <c r="E34" s="7">
         <f t="shared" si="2"/>
         <v>4975</v>
       </c>
     </row>
-    <row r="34" spans="2:5">
-      <c r="B34" t="s">
+    <row r="35" spans="2:5">
+      <c r="B35" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C34" s="2">
+      <c r="C35" s="6">
         <v>5</v>
       </c>
-      <c r="D34" s="2">
+      <c r="D35" s="6">
         <v>2500</v>
       </c>
-      <c r="E34" s="3">
+      <c r="E35" s="7">
         <f t="shared" si="2"/>
         <v>12500</v>
       </c>
     </row>
-    <row r="35" spans="2:5">
-      <c r="B35" s="4" t="s">
+    <row r="36" spans="2:5">
+      <c r="B36" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="5">
+      <c r="C36" s="9">
         <v>6</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D36" s="6">
         <v>3500</v>
       </c>
-      <c r="E35" s="3">
+      <c r="E36" s="7">
         <f t="shared" si="2"/>
         <v>21000</v>
       </c>
     </row>
-    <row r="36" spans="2:5">
-      <c r="B36" s="4" t="s">
+    <row r="37" spans="2:5">
+      <c r="B37" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C36">
+      <c r="C37" s="9">
         <v>6</v>
       </c>
-      <c r="D36">
+      <c r="D37" s="9">
         <v>15000</v>
       </c>
-      <c r="E36" s="3">
+      <c r="E37" s="9">
         <f t="shared" si="2"/>
         <v>90000</v>
       </c>
     </row>
-    <row r="37" spans="2:5">
-      <c r="B37" t="s">
+    <row r="38" spans="2:5">
+      <c r="B38" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C37" s="2">
+      <c r="C38" s="6">
         <v>20</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D38" s="6">
         <v>199</v>
       </c>
-      <c r="E37" s="3">
+      <c r="E38" s="7">
         <f t="shared" si="2"/>
         <v>3980</v>
       </c>
     </row>
-    <row r="38" spans="2:5">
-      <c r="B38" t="s">
+    <row r="39" spans="2:5">
+      <c r="B39" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C38" s="3">
+      <c r="C39" s="7">
         <v>10</v>
       </c>
-      <c r="D38" s="3">
+      <c r="D39" s="7">
         <v>499</v>
       </c>
-      <c r="E38" s="3">
+      <c r="E39" s="7">
         <f t="shared" si="2"/>
         <v>4990</v>
       </c>
     </row>
-    <row r="39" spans="2:5">
-      <c r="B39" t="s">
+    <row r="40" spans="2:5">
+      <c r="B40" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C39" s="3">
+      <c r="C40" s="7">
         <v>10</v>
       </c>
-      <c r="D39" s="3">
+      <c r="D40" s="7">
         <v>799</v>
       </c>
-      <c r="E39" s="3">
+      <c r="E40" s="7">
         <f t="shared" si="2"/>
         <v>7990</v>
       </c>
     </row>
-    <row r="40" spans="2:5">
-      <c r="B40" t="s">
+    <row r="41" spans="2:5">
+      <c r="B41" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C40" s="2">
+      <c r="C41" s="6">
         <v>12</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D41" s="6">
         <v>1399</v>
       </c>
-      <c r="E40" s="3">
+      <c r="E41" s="7">
         <f t="shared" si="2"/>
         <v>16788</v>
       </c>
     </row>
-    <row r="41" spans="2:5">
-      <c r="B41" t="s">
+    <row r="42" spans="2:5">
+      <c r="B42" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C41" s="3">
+      <c r="C42" s="7">
         <v>2</v>
       </c>
-      <c r="D41" s="3">
+      <c r="D42" s="7">
         <v>15000</v>
       </c>
-      <c r="E41" s="3">
+      <c r="E42" s="7">
         <f t="shared" si="2"/>
         <v>30000</v>
       </c>
     </row>
-    <row r="42" spans="3:5">
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
-    </row>
-    <row r="43" spans="3:5">
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
+    <row r="43" spans="2:5">
+      <c r="B43" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C43" s="6">
+        <v>50</v>
+      </c>
+      <c r="D43" s="6">
+        <v>125</v>
+      </c>
+      <c r="E43" s="7">
+        <f t="shared" si="2"/>
+        <v>6250</v>
+      </c>
     </row>
     <row r="44" spans="3:5">
-      <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
-      <c r="E44" s="3"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
     </row>
     <row r="45" spans="3:5">
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
     </row>
     <row r="46" spans="3:5">
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
     </row>
     <row r="47" spans="3:5">
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-    </row>
-    <row r="48" spans="3:5">
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
-    </row>
-    <row r="49" spans="3:5">
-      <c r="C49" s="3"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
-    </row>
-    <row r="50" spans="3:5">
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+    </row>
+    <row r="48" spans="2:5">
+      <c r="B48" t="s">
+        <v>39</v>
+      </c>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+    </row>
+    <row r="49" spans="2:5">
+      <c r="B49" t="s">
+        <v>40</v>
+      </c>
+      <c r="C49" s="10">
+        <v>57000</v>
+      </c>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+    </row>
+    <row r="50" spans="2:5">
+      <c r="B50" t="s">
+        <v>41</v>
+      </c>
+      <c r="C50" s="10">
+        <v>171000</v>
+      </c>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
     </row>
     <row r="51" spans="3:5">
-      <c r="C51" s="3"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="3"/>
+      <c r="C51" s="10">
+        <f>SUM(C49:C50)</f>
+        <v>228000</v>
+      </c>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
     </row>
     <row r="52" spans="3:5">
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-    </row>
-    <row r="53" spans="3:5">
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="10"/>
+    </row>
+    <row r="53" spans="2:5">
+      <c r="B53" t="s">
+        <v>39</v>
+      </c>
+      <c r="C53" s="10"/>
+      <c r="D53" s="10"/>
+      <c r="E53" s="10"/>
+    </row>
+    <row r="54" spans="2:3">
+      <c r="B54" t="s">
+        <v>40</v>
+      </c>
+      <c r="C54" s="10">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="55" spans="2:3">
+      <c r="B55" t="s">
+        <v>41</v>
+      </c>
+      <c r="C55" s="10">
+        <v>360000</v>
+      </c>
+    </row>
+    <row r="56" spans="3:3">
+      <c r="C56" s="10">
+        <f>SUM(C54:C55)</f>
+        <v>460000</v>
+      </c>
+    </row>
+    <row r="58" spans="2:3">
+      <c r="B58" t="s">
+        <v>42</v>
+      </c>
+      <c r="C58" s="10">
+        <v>22000</v>
+      </c>
+    </row>
+    <row r="60" spans="3:3">
+      <c r="C60" s="10">
+        <f>C51+C56+C58</f>
+        <v>710000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="7"/>
+  <cols>
+    <col min="3" max="3" width="40.875" customWidth="1"/>
+    <col min="4" max="11" width="11.5625" customWidth="1"/>
+    <col min="13" max="13" width="63.6875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="2">
+        <v>4500</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2">
+        <v>500</v>
+      </c>
+      <c r="H2" s="2">
+        <f>25*2*2000/100</f>
+        <v>1000</v>
+      </c>
+      <c r="I2" s="2">
+        <v>900</v>
+      </c>
+      <c r="J2" s="2">
+        <f>SUM(G2:I2)</f>
+        <v>2400</v>
+      </c>
+      <c r="K2" s="2">
+        <f>D2-J2</f>
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1500</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2">
+        <v>500</v>
+      </c>
+      <c r="H3" s="2">
+        <f>30*2*2000/100</f>
+        <v>1200</v>
+      </c>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2">
+        <f>SUM(G3:I3)</f>
+        <v>1700</v>
+      </c>
+      <c r="K3" s="2">
+        <f>D3-J3</f>
+        <v>-200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="2">
+        <v>5000</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2">
+        <v>800</v>
+      </c>
+      <c r="H4" s="2">
+        <f>25*3*1700/100</f>
+        <v>1275</v>
+      </c>
+      <c r="I4" s="2">
+        <v>600</v>
+      </c>
+      <c r="J4" s="2">
+        <f>SUM(G4:I4)</f>
+        <v>2675</v>
+      </c>
+      <c r="K4" s="2">
+        <f>D4-J4</f>
+        <v>2325</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2">
+        <v>500</v>
+      </c>
+      <c r="H5" s="2">
+        <f>15*2*1700/100</f>
+        <v>510</v>
+      </c>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2">
+        <f>SUM(G5:I5)</f>
+        <v>1010</v>
+      </c>
+      <c r="K5" s="2">
+        <f>D5-J5</f>
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="6" spans="4:13">
+      <c r="D6" s="3">
+        <f>SUM(D2:D5)</f>
+        <v>12000</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="3">
+        <f>SUM(K2:K5)</f>
+        <v>4215</v>
+      </c>
+      <c r="L6" s="1">
+        <f>K6/5</f>
+        <v>843</v>
+      </c>
+      <c r="M6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="4:6">
+      <c r="D7" s="3">
+        <f>D6*50</f>
+        <v>600000</v>
+      </c>
+      <c r="E7" s="3">
+        <v>50</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="4:6">
+      <c r="D8" s="3">
+        <f>D6*1000</f>
+        <v>12000000</v>
+      </c>
+      <c r="E8" s="3">
+        <v>1000</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>58</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>